<commit_message>
Generate data for office type
</commit_message>
<xml_diff>
--- a/hardware/bom.xlsx
+++ b/hardware/bom.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Liam\Desktop\Projects\room-occupancy\hardware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B40E9921-6CEF-4BEE-8B40-A22774FB67FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{623628CE-869B-4F4E-B702-EC8BEF5EB81F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{FB4A3F76-8793-422F-B4D4-A7C3F2C8A7F2}"/>
   </bookViews>
@@ -68,9 +68,6 @@
     <t>KOSTEN</t>
   </si>
   <si>
-    <t>EEMB LiPo 2700 mA</t>
-  </si>
-  <si>
     <t>Akku</t>
   </si>
   <si>
@@ -78,6 +75,9 @@
   </si>
   <si>
     <t>Waveshare 7.5 mit HAT v2</t>
+  </si>
+  <si>
+    <t>EEMB LiPo 3700 mA</t>
   </si>
 </sst>
 </file>
@@ -501,10 +501,10 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" t="s">
         <v>10</v>
-      </c>
-      <c r="B2" t="s">
-        <v>11</v>
       </c>
       <c r="C2">
         <v>13</v>
@@ -523,7 +523,7 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B3" t="s">
         <v>5</v>
@@ -544,7 +544,7 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
         <v>7</v>

</xml_diff>